<commit_message>
Doi phan loai FIBond repo sang 4 nhom theo chan truoc x Gross so sanh
Thay nhi phan di vay/cho vay bang 4 nhom: Cho vay tien, Vay bond, Di vay
tien, Cho vay bong - theo (chan nao thanh toan truoc) x (Gross ben nao lon
hon). Cap nhat script ghep cap, script xuat xlsx (chinh thuc hoa vao
bond/tools/), file Excel da tao lai, va docs.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013YvXH6YGUnvcjZtzC6iCb9
</commit_message>
<xml_diff>
--- a/bond/Deal_FIBond_Repo_20260824.xlsx
+++ b/bond/Deal_FIBond_Repo_20260824.xlsx
@@ -604,7 +604,7 @@
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>Reverse Repo (cho vay)</t>
+          <t>Cho vay tien</t>
         </is>
       </c>
       <c r="L2" s="5" t="n">
@@ -676,7 +676,7 @@
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>Reverse Repo (cho vay)</t>
+          <t>Cho vay tien</t>
         </is>
       </c>
       <c r="L3" s="5" t="n">
@@ -748,7 +748,7 @@
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>Reverse Repo (cho vay)</t>
+          <t>Cho vay tien</t>
         </is>
       </c>
       <c r="L4" s="5" t="n">
@@ -820,7 +820,7 @@
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>Reverse Repo (cho vay)</t>
+          <t>Cho vay tien</t>
         </is>
       </c>
       <c r="L5" s="5" t="n">
@@ -892,7 +892,7 @@
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>Reverse Repo (cho vay)</t>
+          <t>Cho vay tien</t>
         </is>
       </c>
       <c r="L6" s="5" t="n">
@@ -964,7 +964,7 @@
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>Reverse Repo (cho vay)</t>
+          <t>Cho vay tien</t>
         </is>
       </c>
       <c r="L7" s="5" t="n">
@@ -1036,7 +1036,7 @@
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>Reverse Repo (cho vay)</t>
+          <t>Cho vay tien</t>
         </is>
       </c>
       <c r="L8" s="5" t="n">
@@ -1108,7 +1108,7 @@
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>Reverse Repo (cho vay)</t>
+          <t>Cho vay tien</t>
         </is>
       </c>
       <c r="L9" s="5" t="n">
@@ -1180,7 +1180,7 @@
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>Reverse Repo (cho vay)</t>
+          <t>Cho vay tien</t>
         </is>
       </c>
       <c r="L10" s="5" t="n">
@@ -1252,7 +1252,7 @@
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>Reverse Repo (cho vay)</t>
+          <t>Cho vay tien</t>
         </is>
       </c>
       <c r="L11" s="5" t="n">
@@ -1324,7 +1324,7 @@
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>Reverse Repo (cho vay)</t>
+          <t>Cho vay tien</t>
         </is>
       </c>
       <c r="L12" s="5" t="n">
@@ -1396,7 +1396,7 @@
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>Reverse Repo (cho vay)</t>
+          <t>Cho vay tien</t>
         </is>
       </c>
       <c r="L13" s="5" t="n">
@@ -1468,7 +1468,7 @@
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>Reverse Repo (cho vay)</t>
+          <t>Cho vay tien</t>
         </is>
       </c>
       <c r="L14" s="5" t="n">
@@ -1540,7 +1540,7 @@
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>Reverse Repo (cho vay)</t>
+          <t>Cho vay tien</t>
         </is>
       </c>
       <c r="L15" s="5" t="n">
@@ -1612,7 +1612,7 @@
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L16" s="5" t="n">
@@ -1684,7 +1684,7 @@
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L17" s="5" t="n">
@@ -1756,7 +1756,7 @@
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L18" s="5" t="n">
@@ -1828,7 +1828,7 @@
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L19" s="5" t="n">
@@ -1900,7 +1900,7 @@
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L20" s="5" t="n">
@@ -1972,7 +1972,7 @@
       </c>
       <c r="K21" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L21" s="5" t="n">
@@ -2044,7 +2044,7 @@
       </c>
       <c r="K22" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L22" s="5" t="n">
@@ -2116,7 +2116,7 @@
       </c>
       <c r="K23" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L23" s="5" t="n">
@@ -2188,7 +2188,7 @@
       </c>
       <c r="K24" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L24" s="5" t="n">
@@ -2260,7 +2260,7 @@
       </c>
       <c r="K25" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L25" s="5" t="n">
@@ -2332,7 +2332,7 @@
       </c>
       <c r="K26" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L26" s="5" t="n">
@@ -2404,7 +2404,7 @@
       </c>
       <c r="K27" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L27" s="5" t="n">
@@ -2476,7 +2476,7 @@
       </c>
       <c r="K28" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L28" s="5" t="n">
@@ -2548,7 +2548,7 @@
       </c>
       <c r="K29" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L29" s="5" t="n">
@@ -2620,7 +2620,7 @@
       </c>
       <c r="K30" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L30" s="5" t="n">
@@ -2692,7 +2692,7 @@
       </c>
       <c r="K31" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L31" s="5" t="n">
@@ -2764,7 +2764,7 @@
       </c>
       <c r="K32" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L32" s="5" t="n">
@@ -2836,7 +2836,7 @@
       </c>
       <c r="K33" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L33" s="5" t="n">
@@ -2908,7 +2908,7 @@
       </c>
       <c r="K34" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L34" s="5" t="n">
@@ -2980,7 +2980,7 @@
       </c>
       <c r="K35" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L35" s="5" t="n">
@@ -3052,7 +3052,7 @@
       </c>
       <c r="K36" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L36" s="5" t="n">
@@ -3124,7 +3124,7 @@
       </c>
       <c r="K37" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L37" s="5" t="n">
@@ -3196,7 +3196,7 @@
       </c>
       <c r="K38" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L38" s="5" t="n">
@@ -3268,7 +3268,7 @@
       </c>
       <c r="K39" s="2" t="inlineStr">
         <is>
-          <t>Reverse Repo (cho vay)</t>
+          <t>Cho vay tien</t>
         </is>
       </c>
       <c r="L39" s="5" t="n">
@@ -3340,7 +3340,7 @@
       </c>
       <c r="K40" s="2" t="inlineStr">
         <is>
-          <t>Reverse Repo (cho vay)</t>
+          <t>Cho vay tien</t>
         </is>
       </c>
       <c r="L40" s="5" t="n">
@@ -3412,7 +3412,7 @@
       </c>
       <c r="K41" s="2" t="inlineStr">
         <is>
-          <t>Reverse Repo (cho vay)</t>
+          <t>Cho vay tien</t>
         </is>
       </c>
       <c r="L41" s="5" t="n">
@@ -3484,7 +3484,7 @@
       </c>
       <c r="K42" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L42" s="5" t="n">
@@ -3556,7 +3556,7 @@
       </c>
       <c r="K43" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L43" s="5" t="n">
@@ -3628,7 +3628,7 @@
       </c>
       <c r="K44" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L44" s="5" t="n">
@@ -3700,7 +3700,7 @@
       </c>
       <c r="K45" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L45" s="5" t="n">
@@ -3772,7 +3772,7 @@
       </c>
       <c r="K46" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L46" s="5" t="n">
@@ -3844,7 +3844,7 @@
       </c>
       <c r="K47" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L47" s="5" t="n">
@@ -3916,7 +3916,7 @@
       </c>
       <c r="K48" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L48" s="5" t="n">
@@ -3988,7 +3988,7 @@
       </c>
       <c r="K49" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L49" s="5" t="n">
@@ -4060,7 +4060,7 @@
       </c>
       <c r="K50" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L50" s="5" t="n">
@@ -4132,7 +4132,7 @@
       </c>
       <c r="K51" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L51" s="5" t="n">
@@ -4204,7 +4204,7 @@
       </c>
       <c r="K52" s="2" t="inlineStr">
         <is>
-          <t>Reverse Repo (cho vay)</t>
+          <t>Cho vay tien</t>
         </is>
       </c>
       <c r="L52" s="5" t="n">
@@ -4276,7 +4276,7 @@
       </c>
       <c r="K53" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L53" s="5" t="n">
@@ -4348,7 +4348,7 @@
       </c>
       <c r="K54" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L54" s="5" t="n">
@@ -4420,7 +4420,7 @@
       </c>
       <c r="K55" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L55" s="5" t="n">
@@ -4631,7 +4631,7 @@
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L2" s="5" t="n">
@@ -4703,7 +4703,7 @@
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L3" s="5" t="n">
@@ -4775,7 +4775,7 @@
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L4" s="5" t="n">
@@ -4847,7 +4847,7 @@
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L5" s="5" t="n">
@@ -4919,7 +4919,7 @@
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L6" s="5" t="n">
@@ -4991,7 +4991,7 @@
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>Reverse Repo (cho vay)</t>
+          <t>Cho vay tien</t>
         </is>
       </c>
       <c r="L7" s="5" t="n">
@@ -5063,7 +5063,7 @@
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>Reverse Repo (cho vay)</t>
+          <t>Cho vay tien</t>
         </is>
       </c>
       <c r="L8" s="5" t="n">
@@ -5135,7 +5135,7 @@
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>Reverse Repo (cho vay)</t>
+          <t>Cho vay tien</t>
         </is>
       </c>
       <c r="L9" s="5" t="n">
@@ -5207,7 +5207,7 @@
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>Reverse Repo (cho vay)</t>
+          <t>Cho vay tien</t>
         </is>
       </c>
       <c r="L10" s="5" t="n">
@@ -5279,7 +5279,7 @@
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>Reverse Repo (cho vay)</t>
+          <t>Cho vay tien</t>
         </is>
       </c>
       <c r="L11" s="5" t="n">
@@ -5351,7 +5351,7 @@
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>Reverse Repo (cho vay)</t>
+          <t>Cho vay tien</t>
         </is>
       </c>
       <c r="L12" s="5" t="n">
@@ -5423,7 +5423,7 @@
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>Reverse Repo (cho vay)</t>
+          <t>Cho vay tien</t>
         </is>
       </c>
       <c r="L13" s="5" t="n">
@@ -5495,7 +5495,7 @@
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>Reverse Repo (cho vay)</t>
+          <t>Cho vay tien</t>
         </is>
       </c>
       <c r="L14" s="5" t="n">
@@ -5567,7 +5567,7 @@
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>Reverse Repo (cho vay)</t>
+          <t>Cho vay tien</t>
         </is>
       </c>
       <c r="L15" s="5" t="n">
@@ -5639,7 +5639,7 @@
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>Reverse Repo (cho vay)</t>
+          <t>Cho vay tien</t>
         </is>
       </c>
       <c r="L16" s="5" t="n">
@@ -5711,7 +5711,7 @@
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>Reverse Repo (cho vay)</t>
+          <t>Cho vay tien</t>
         </is>
       </c>
       <c r="L17" s="5" t="n">
@@ -5783,7 +5783,7 @@
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>Reverse Repo (cho vay)</t>
+          <t>Cho vay tien</t>
         </is>
       </c>
       <c r="L18" s="5" t="n">
@@ -5855,7 +5855,7 @@
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>Reverse Repo (cho vay)</t>
+          <t>Cho vay tien</t>
         </is>
       </c>
       <c r="L19" s="5" t="n">
@@ -5927,7 +5927,7 @@
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>Reverse Repo (cho vay)</t>
+          <t>Cho vay tien</t>
         </is>
       </c>
       <c r="L20" s="5" t="n">
@@ -5999,7 +5999,7 @@
       </c>
       <c r="K21" s="2" t="inlineStr">
         <is>
-          <t>Reverse Repo (cho vay)</t>
+          <t>Cho vay tien</t>
         </is>
       </c>
       <c r="L21" s="5" t="n">
@@ -6071,7 +6071,7 @@
       </c>
       <c r="K22" s="2" t="inlineStr">
         <is>
-          <t>Reverse Repo (cho vay)</t>
+          <t>Cho vay tien</t>
         </is>
       </c>
       <c r="L22" s="5" t="n">
@@ -6143,7 +6143,7 @@
       </c>
       <c r="K23" s="2" t="inlineStr">
         <is>
-          <t>Reverse Repo (cho vay)</t>
+          <t>Cho vay tien</t>
         </is>
       </c>
       <c r="L23" s="5" t="n">
@@ -6215,7 +6215,7 @@
       </c>
       <c r="K24" s="2" t="inlineStr">
         <is>
-          <t>Reverse Repo (cho vay)</t>
+          <t>Cho vay tien</t>
         </is>
       </c>
       <c r="L24" s="5" t="n">
@@ -6287,7 +6287,7 @@
       </c>
       <c r="K25" s="2" t="inlineStr">
         <is>
-          <t>Reverse Repo (cho vay)</t>
+          <t>Cho vay tien</t>
         </is>
       </c>
       <c r="L25" s="5" t="n">
@@ -6359,7 +6359,7 @@
       </c>
       <c r="K26" s="2" t="inlineStr">
         <is>
-          <t>Reverse Repo (cho vay)</t>
+          <t>Cho vay tien</t>
         </is>
       </c>
       <c r="L26" s="5" t="n">
@@ -6431,7 +6431,7 @@
       </c>
       <c r="K27" s="2" t="inlineStr">
         <is>
-          <t>Reverse Repo (cho vay)</t>
+          <t>Cho vay tien</t>
         </is>
       </c>
       <c r="L27" s="5" t="n">
@@ -6503,7 +6503,7 @@
       </c>
       <c r="K28" s="2" t="inlineStr">
         <is>
-          <t>Reverse Repo (cho vay)</t>
+          <t>Cho vay tien</t>
         </is>
       </c>
       <c r="L28" s="5" t="n">
@@ -6575,7 +6575,7 @@
       </c>
       <c r="K29" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L29" s="5" t="n">
@@ -6647,7 +6647,7 @@
       </c>
       <c r="K30" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L30" s="5" t="n">
@@ -6719,7 +6719,7 @@
       </c>
       <c r="K31" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L31" s="5" t="n">
@@ -6791,7 +6791,7 @@
       </c>
       <c r="K32" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L32" s="5" t="n">
@@ -6863,7 +6863,7 @@
       </c>
       <c r="K33" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L33" s="5" t="n">
@@ -6935,7 +6935,7 @@
       </c>
       <c r="K34" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L34" s="5" t="n">
@@ -7007,7 +7007,7 @@
       </c>
       <c r="K35" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L35" s="5" t="n">
@@ -7079,7 +7079,7 @@
       </c>
       <c r="K36" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L36" s="5" t="n">
@@ -7151,7 +7151,7 @@
       </c>
       <c r="K37" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L37" s="5" t="n">
@@ -7223,7 +7223,7 @@
       </c>
       <c r="K38" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L38" s="5" t="n">
@@ -7295,7 +7295,7 @@
       </c>
       <c r="K39" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L39" s="5" t="n">
@@ -7367,7 +7367,7 @@
       </c>
       <c r="K40" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L40" s="5" t="n">
@@ -7439,7 +7439,7 @@
       </c>
       <c r="K41" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L41" s="5" t="n">
@@ -7511,7 +7511,7 @@
       </c>
       <c r="K42" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L42" s="5" t="n">
@@ -7583,7 +7583,7 @@
       </c>
       <c r="K43" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L43" s="5" t="n">
@@ -7655,7 +7655,7 @@
       </c>
       <c r="K44" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L44" s="5" t="n">
@@ -7727,7 +7727,7 @@
       </c>
       <c r="K45" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L45" s="5" t="n">
@@ -7799,7 +7799,7 @@
       </c>
       <c r="K46" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L46" s="5" t="n">
@@ -7871,7 +7871,7 @@
       </c>
       <c r="K47" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L47" s="5" t="n">
@@ -7943,7 +7943,7 @@
       </c>
       <c r="K48" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L48" s="5" t="n">
@@ -8015,7 +8015,7 @@
       </c>
       <c r="K49" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L49" s="5" t="n">
@@ -8087,7 +8087,7 @@
       </c>
       <c r="K50" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L50" s="5" t="n">
@@ -8159,7 +8159,7 @@
       </c>
       <c r="K51" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L51" s="5" t="n">
@@ -8231,7 +8231,7 @@
       </c>
       <c r="K52" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L52" s="5" t="n">
@@ -8303,7 +8303,7 @@
       </c>
       <c r="K53" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L53" s="5" t="n">
@@ -8375,7 +8375,7 @@
       </c>
       <c r="K54" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L54" s="5" t="n">
@@ -8447,7 +8447,7 @@
       </c>
       <c r="K55" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L55" s="5" t="n">
@@ -8519,7 +8519,7 @@
       </c>
       <c r="K56" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L56" s="5" t="n">
@@ -8591,7 +8591,7 @@
       </c>
       <c r="K57" s="2" t="inlineStr">
         <is>
-          <t>Reverse Repo (cho vay)</t>
+          <t>Cho vay tien</t>
         </is>
       </c>
       <c r="L57" s="5" t="n">
@@ -8663,7 +8663,7 @@
       </c>
       <c r="K58" s="2" t="inlineStr">
         <is>
-          <t>Reverse Repo (cho vay)</t>
+          <t>Cho vay tien</t>
         </is>
       </c>
       <c r="L58" s="5" t="n">
@@ -8735,7 +8735,7 @@
       </c>
       <c r="K59" s="2" t="inlineStr">
         <is>
-          <t>Reverse Repo (cho vay)</t>
+          <t>Cho vay tien</t>
         </is>
       </c>
       <c r="L59" s="5" t="n">
@@ -8807,7 +8807,7 @@
       </c>
       <c r="K60" s="2" t="inlineStr">
         <is>
-          <t>Reverse Repo (cho vay)</t>
+          <t>Cho vay tien</t>
         </is>
       </c>
       <c r="L60" s="5" t="n">
@@ -8879,7 +8879,7 @@
       </c>
       <c r="K61" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L61" s="5" t="n">
@@ -8951,7 +8951,7 @@
       </c>
       <c r="K62" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L62" s="5" t="n">
@@ -9023,7 +9023,7 @@
       </c>
       <c r="K63" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L63" s="5" t="n">
@@ -9095,7 +9095,7 @@
       </c>
       <c r="K64" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L64" s="5" t="n">
@@ -9167,7 +9167,7 @@
       </c>
       <c r="K65" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L65" s="5" t="n">
@@ -9239,7 +9239,7 @@
       </c>
       <c r="K66" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L66" s="5" t="n">
@@ -9311,7 +9311,7 @@
       </c>
       <c r="K67" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L67" s="5" t="n">
@@ -9383,7 +9383,7 @@
       </c>
       <c r="K68" s="2" t="inlineStr">
         <is>
-          <t>Reverse Repo (cho vay)</t>
+          <t>Cho vay tien</t>
         </is>
       </c>
       <c r="L68" s="5" t="n">
@@ -9455,7 +9455,7 @@
       </c>
       <c r="K69" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L69" s="5" t="n">
@@ -9527,7 +9527,7 @@
       </c>
       <c r="K70" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L70" s="5" t="n">
@@ -9599,7 +9599,7 @@
       </c>
       <c r="K71" s="2" t="inlineStr">
         <is>
-          <t>Reverse Repo (cho vay)</t>
+          <t>Cho vay tien</t>
         </is>
       </c>
       <c r="L71" s="5" t="n">
@@ -9671,7 +9671,7 @@
       </c>
       <c r="K72" s="2" t="inlineStr">
         <is>
-          <t>Reverse Repo (cho vay)</t>
+          <t>Cho vay tien</t>
         </is>
       </c>
       <c r="L72" s="5" t="n">
@@ -9743,7 +9743,7 @@
       </c>
       <c r="K73" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L73" s="5" t="n">
@@ -9815,7 +9815,7 @@
       </c>
       <c r="K74" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L74" s="5" t="n">
@@ -9887,7 +9887,7 @@
       </c>
       <c r="K75" s="2" t="inlineStr">
         <is>
-          <t>Reverse Repo (cho vay)</t>
+          <t>Cho vay tien</t>
         </is>
       </c>
       <c r="L75" s="5" t="n">
@@ -9959,7 +9959,7 @@
       </c>
       <c r="K76" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L76" s="5" t="n">
@@ -10031,7 +10031,7 @@
       </c>
       <c r="K77" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L77" s="5" t="n">
@@ -10103,7 +10103,7 @@
       </c>
       <c r="K78" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L78" s="5" t="n">
@@ -10175,7 +10175,7 @@
       </c>
       <c r="K79" s="2" t="inlineStr">
         <is>
-          <t>Reverse Repo (cho vay)</t>
+          <t>Cho vay tien</t>
         </is>
       </c>
       <c r="L79" s="5" t="n">
@@ -10247,7 +10247,7 @@
       </c>
       <c r="K80" s="2" t="inlineStr">
         <is>
-          <t>Reverse Repo (cho vay)</t>
+          <t>Cho vay tien</t>
         </is>
       </c>
       <c r="L80" s="5" t="n">
@@ -10319,7 +10319,7 @@
       </c>
       <c r="K81" s="2" t="inlineStr">
         <is>
-          <t>Reverse Repo (cho vay)</t>
+          <t>Cho vay tien</t>
         </is>
       </c>
       <c r="L81" s="5" t="n">
@@ -10391,7 +10391,7 @@
       </c>
       <c r="K82" s="2" t="inlineStr">
         <is>
-          <t>Reverse Repo (cho vay)</t>
+          <t>Cho vay tien</t>
         </is>
       </c>
       <c r="L82" s="5" t="n">
@@ -10463,7 +10463,7 @@
       </c>
       <c r="K83" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L83" s="5" t="n">
@@ -10535,7 +10535,7 @@
       </c>
       <c r="K84" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L84" s="5" t="n">
@@ -10607,7 +10607,7 @@
       </c>
       <c r="K85" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L85" s="5" t="n">
@@ -10679,7 +10679,7 @@
       </c>
       <c r="K86" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L86" s="5" t="n">
@@ -10751,7 +10751,7 @@
       </c>
       <c r="K87" s="2" t="inlineStr">
         <is>
-          <t>Reverse Repo (cho vay)</t>
+          <t>Cho vay tien</t>
         </is>
       </c>
       <c r="L87" s="5" t="n">
@@ -10823,7 +10823,7 @@
       </c>
       <c r="K88" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L88" s="5" t="n">
@@ -10895,7 +10895,7 @@
       </c>
       <c r="K89" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L89" s="5" t="n">
@@ -10967,7 +10967,7 @@
       </c>
       <c r="K90" s="2" t="inlineStr">
         <is>
-          <t>Reverse Repo (cho vay)</t>
+          <t>Cho vay tien</t>
         </is>
       </c>
       <c r="L90" s="5" t="n">
@@ -11039,7 +11039,7 @@
       </c>
       <c r="K91" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L91" s="5" t="n">
@@ -11111,7 +11111,7 @@
       </c>
       <c r="K92" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L92" s="5" t="n">
@@ -11183,7 +11183,7 @@
       </c>
       <c r="K93" s="2" t="inlineStr">
         <is>
-          <t>Reverse Repo (cho vay)</t>
+          <t>Cho vay tien</t>
         </is>
       </c>
       <c r="L93" s="5" t="n">
@@ -11255,7 +11255,7 @@
       </c>
       <c r="K94" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L94" s="5" t="n">
@@ -11327,7 +11327,7 @@
       </c>
       <c r="K95" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L95" s="5" t="n">
@@ -11399,7 +11399,7 @@
       </c>
       <c r="K96" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L96" s="5" t="n">
@@ -11471,7 +11471,7 @@
       </c>
       <c r="K97" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L97" s="5" t="n">
@@ -11543,7 +11543,7 @@
       </c>
       <c r="K98" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L98" s="5" t="n">
@@ -11615,7 +11615,7 @@
       </c>
       <c r="K99" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L99" s="5" t="n">
@@ -11687,7 +11687,7 @@
       </c>
       <c r="K100" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L100" s="5" t="n">
@@ -11759,7 +11759,7 @@
       </c>
       <c r="K101" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L101" s="5" t="n">
@@ -11831,7 +11831,7 @@
       </c>
       <c r="K102" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L102" s="5" t="n">
@@ -11903,7 +11903,7 @@
       </c>
       <c r="K103" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L103" s="5" t="n">
@@ -11975,7 +11975,7 @@
       </c>
       <c r="K104" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L104" s="5" t="n">
@@ -12047,7 +12047,7 @@
       </c>
       <c r="K105" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L105" s="5" t="n">
@@ -12119,7 +12119,7 @@
       </c>
       <c r="K106" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L106" s="5" t="n">
@@ -12191,7 +12191,7 @@
       </c>
       <c r="K107" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L107" s="5" t="n">
@@ -12263,7 +12263,7 @@
       </c>
       <c r="K108" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L108" s="5" t="n">
@@ -12335,7 +12335,7 @@
       </c>
       <c r="K109" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L109" s="5" t="n">
@@ -12407,7 +12407,7 @@
       </c>
       <c r="K110" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L110" s="5" t="n">
@@ -12479,7 +12479,7 @@
       </c>
       <c r="K111" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L111" s="5" t="n">
@@ -12551,7 +12551,7 @@
       </c>
       <c r="K112" s="2" t="inlineStr">
         <is>
-          <t>Reverse Repo (cho vay)</t>
+          <t>Cho vay tien</t>
         </is>
       </c>
       <c r="L112" s="5" t="n">
@@ -12623,7 +12623,7 @@
       </c>
       <c r="K113" s="2" t="inlineStr">
         <is>
-          <t>Reverse Repo (cho vay)</t>
+          <t>Cho vay tien</t>
         </is>
       </c>
       <c r="L113" s="5" t="n">
@@ -12695,7 +12695,7 @@
       </c>
       <c r="K114" s="2" t="inlineStr">
         <is>
-          <t>Reverse Repo (cho vay)</t>
+          <t>Cho vay tien</t>
         </is>
       </c>
       <c r="L114" s="5" t="n">
@@ -12767,7 +12767,7 @@
       </c>
       <c r="K115" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L115" s="5" t="n">
@@ -12839,7 +12839,7 @@
       </c>
       <c r="K116" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L116" s="5" t="n">
@@ -12911,7 +12911,7 @@
       </c>
       <c r="K117" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L117" s="5" t="n">
@@ -12983,7 +12983,7 @@
       </c>
       <c r="K118" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L118" s="5" t="n">
@@ -13055,7 +13055,7 @@
       </c>
       <c r="K119" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L119" s="5" t="n">
@@ -13127,7 +13127,7 @@
       </c>
       <c r="K120" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L120" s="5" t="n">
@@ -13199,7 +13199,7 @@
       </c>
       <c r="K121" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L121" s="5" t="n">
@@ -13271,7 +13271,7 @@
       </c>
       <c r="K122" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L122" s="5" t="n">
@@ -13343,7 +13343,7 @@
       </c>
       <c r="K123" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L123" s="5" t="n">
@@ -13415,7 +13415,7 @@
       </c>
       <c r="K124" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L124" s="5" t="n">
@@ -13487,7 +13487,7 @@
       </c>
       <c r="K125" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L125" s="5" t="n">
@@ -13559,7 +13559,7 @@
       </c>
       <c r="K126" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L126" s="5" t="n">
@@ -13631,7 +13631,7 @@
       </c>
       <c r="K127" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L127" s="5" t="n">
@@ -13703,7 +13703,7 @@
       </c>
       <c r="K128" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L128" s="5" t="n">
@@ -13775,7 +13775,7 @@
       </c>
       <c r="K129" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L129" s="5" t="n">
@@ -13847,7 +13847,7 @@
       </c>
       <c r="K130" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L130" s="5" t="n">
@@ -13919,7 +13919,7 @@
       </c>
       <c r="K131" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L131" s="5" t="n">
@@ -13991,7 +13991,7 @@
       </c>
       <c r="K132" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L132" s="5" t="n">
@@ -14063,7 +14063,7 @@
       </c>
       <c r="K133" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L133" s="5" t="n">
@@ -14135,7 +14135,7 @@
       </c>
       <c r="K134" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L134" s="5" t="n">
@@ -14207,7 +14207,7 @@
       </c>
       <c r="K135" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L135" s="5" t="n">
@@ -14279,7 +14279,7 @@
       </c>
       <c r="K136" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L136" s="5" t="n">
@@ -14351,7 +14351,7 @@
       </c>
       <c r="K137" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L137" s="5" t="n">
@@ -14423,7 +14423,7 @@
       </c>
       <c r="K138" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L138" s="5" t="n">
@@ -14495,7 +14495,7 @@
       </c>
       <c r="K139" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L139" s="5" t="n">
@@ -14567,7 +14567,7 @@
       </c>
       <c r="K140" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L140" s="5" t="n">
@@ -14639,7 +14639,7 @@
       </c>
       <c r="K141" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L141" s="5" t="n">
@@ -14711,7 +14711,7 @@
       </c>
       <c r="K142" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L142" s="5" t="n">
@@ -14783,7 +14783,7 @@
       </c>
       <c r="K143" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L143" s="5" t="n">
@@ -14855,7 +14855,7 @@
       </c>
       <c r="K144" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L144" s="5" t="n">
@@ -14927,7 +14927,7 @@
       </c>
       <c r="K145" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L145" s="5" t="n">
@@ -14999,7 +14999,7 @@
       </c>
       <c r="K146" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L146" s="5" t="n">
@@ -15071,7 +15071,7 @@
       </c>
       <c r="K147" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L147" s="5" t="n">
@@ -15143,7 +15143,7 @@
       </c>
       <c r="K148" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L148" s="5" t="n">
@@ -15215,7 +15215,7 @@
       </c>
       <c r="K149" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L149" s="5" t="n">
@@ -15287,7 +15287,7 @@
       </c>
       <c r="K150" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L150" s="5" t="n">
@@ -15359,7 +15359,7 @@
       </c>
       <c r="K151" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L151" s="5" t="n">
@@ -15431,7 +15431,7 @@
       </c>
       <c r="K152" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L152" s="5" t="n">
@@ -15503,7 +15503,7 @@
       </c>
       <c r="K153" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L153" s="5" t="n">
@@ -15575,7 +15575,7 @@
       </c>
       <c r="K154" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L154" s="5" t="n">
@@ -15647,7 +15647,7 @@
       </c>
       <c r="K155" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L155" s="5" t="n">
@@ -15719,7 +15719,7 @@
       </c>
       <c r="K156" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L156" s="5" t="n">
@@ -15791,7 +15791,7 @@
       </c>
       <c r="K157" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L157" s="5" t="n">
@@ -15863,7 +15863,7 @@
       </c>
       <c r="K158" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L158" s="5" t="n">
@@ -15935,7 +15935,7 @@
       </c>
       <c r="K159" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L159" s="5" t="n">
@@ -16007,7 +16007,7 @@
       </c>
       <c r="K160" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L160" s="5" t="n">
@@ -16079,7 +16079,7 @@
       </c>
       <c r="K161" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L161" s="5" t="n">
@@ -16151,7 +16151,7 @@
       </c>
       <c r="K162" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L162" s="5" t="n">
@@ -16223,7 +16223,7 @@
       </c>
       <c r="K163" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L163" s="5" t="n">
@@ -16295,7 +16295,7 @@
       </c>
       <c r="K164" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L164" s="5" t="n">
@@ -16367,7 +16367,7 @@
       </c>
       <c r="K165" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L165" s="5" t="n">
@@ -16439,7 +16439,7 @@
       </c>
       <c r="K166" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L166" s="5" t="n">
@@ -16511,7 +16511,7 @@
       </c>
       <c r="K167" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L167" s="5" t="n">
@@ -16583,7 +16583,7 @@
       </c>
       <c r="K168" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L168" s="5" t="n">
@@ -16655,7 +16655,7 @@
       </c>
       <c r="K169" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L169" s="5" t="n">
@@ -16727,7 +16727,7 @@
       </c>
       <c r="K170" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L170" s="5" t="n">
@@ -16799,7 +16799,7 @@
       </c>
       <c r="K171" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L171" s="5" t="n">
@@ -16871,7 +16871,7 @@
       </c>
       <c r="K172" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L172" s="5" t="n">
@@ -16943,7 +16943,7 @@
       </c>
       <c r="K173" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L173" s="5" t="n">
@@ -17015,7 +17015,7 @@
       </c>
       <c r="K174" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L174" s="5" t="n">
@@ -17087,7 +17087,7 @@
       </c>
       <c r="K175" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L175" s="5" t="n">
@@ -17159,7 +17159,7 @@
       </c>
       <c r="K176" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L176" s="5" t="n">
@@ -17231,7 +17231,7 @@
       </c>
       <c r="K177" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L177" s="5" t="n">
@@ -17303,7 +17303,7 @@
       </c>
       <c r="K178" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L178" s="5" t="n">
@@ -17375,7 +17375,7 @@
       </c>
       <c r="K179" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L179" s="5" t="n">
@@ -17447,7 +17447,7 @@
       </c>
       <c r="K180" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L180" s="5" t="n">
@@ -17519,7 +17519,7 @@
       </c>
       <c r="K181" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L181" s="5" t="n">
@@ -17591,7 +17591,7 @@
       </c>
       <c r="K182" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L182" s="5" t="n">
@@ -17663,7 +17663,7 @@
       </c>
       <c r="K183" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L183" s="5" t="n">
@@ -17735,7 +17735,7 @@
       </c>
       <c r="K184" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L184" s="5" t="n">
@@ -17807,7 +17807,7 @@
       </c>
       <c r="K185" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L185" s="5" t="n">
@@ -17879,7 +17879,7 @@
       </c>
       <c r="K186" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L186" s="5" t="n">
@@ -17951,7 +17951,7 @@
       </c>
       <c r="K187" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L187" s="5" t="n">
@@ -18023,7 +18023,7 @@
       </c>
       <c r="K188" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L188" s="5" t="n">
@@ -18095,7 +18095,7 @@
       </c>
       <c r="K189" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L189" s="5" t="n">
@@ -18167,7 +18167,7 @@
       </c>
       <c r="K190" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L190" s="5" t="n">
@@ -18239,7 +18239,7 @@
       </c>
       <c r="K191" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L191" s="5" t="n">
@@ -18311,7 +18311,7 @@
       </c>
       <c r="K192" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L192" s="5" t="n">
@@ -18383,7 +18383,7 @@
       </c>
       <c r="K193" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L193" s="5" t="n">
@@ -18455,7 +18455,7 @@
       </c>
       <c r="K194" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L194" s="5" t="n">
@@ -18527,7 +18527,7 @@
       </c>
       <c r="K195" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L195" s="5" t="n">
@@ -18599,7 +18599,7 @@
       </c>
       <c r="K196" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L196" s="5" t="n">
@@ -18671,7 +18671,7 @@
       </c>
       <c r="K197" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L197" s="5" t="n">
@@ -18743,7 +18743,7 @@
       </c>
       <c r="K198" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L198" s="5" t="n">
@@ -18815,7 +18815,7 @@
       </c>
       <c r="K199" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L199" s="5" t="n">
@@ -18887,7 +18887,7 @@
       </c>
       <c r="K200" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L200" s="5" t="n">
@@ -18959,7 +18959,7 @@
       </c>
       <c r="K201" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L201" s="5" t="n">
@@ -19031,7 +19031,7 @@
       </c>
       <c r="K202" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L202" s="5" t="n">
@@ -19103,7 +19103,7 @@
       </c>
       <c r="K203" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L203" s="5" t="n">
@@ -19175,7 +19175,7 @@
       </c>
       <c r="K204" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L204" s="5" t="n">
@@ -19247,7 +19247,7 @@
       </c>
       <c r="K205" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L205" s="5" t="n">
@@ -19319,7 +19319,7 @@
       </c>
       <c r="K206" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Di vay tien</t>
         </is>
       </c>
       <c r="L206" s="5" t="n">
@@ -19391,7 +19391,7 @@
       </c>
       <c r="K207" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L207" s="5" t="n">
@@ -19463,7 +19463,7 @@
       </c>
       <c r="K208" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L208" s="5" t="n">
@@ -19535,7 +19535,7 @@
       </c>
       <c r="K209" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L209" s="5" t="n">
@@ -19607,7 +19607,7 @@
       </c>
       <c r="K210" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L210" s="5" t="n">
@@ -19679,7 +19679,7 @@
       </c>
       <c r="K211" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L211" s="5" t="n">
@@ -19751,7 +19751,7 @@
       </c>
       <c r="K212" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L212" s="5" t="n">
@@ -19823,7 +19823,7 @@
       </c>
       <c r="K213" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L213" s="5" t="n">
@@ -19895,7 +19895,7 @@
       </c>
       <c r="K214" s="2" t="inlineStr">
         <is>
-          <t>Reverse Repo (cho vay)</t>
+          <t>Cho vay tien</t>
         </is>
       </c>
       <c r="L214" s="5" t="n">
@@ -19967,7 +19967,7 @@
       </c>
       <c r="K215" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L215" s="5" t="n">
@@ -20039,7 +20039,7 @@
       </c>
       <c r="K216" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L216" s="5" t="n">
@@ -20111,7 +20111,7 @@
       </c>
       <c r="K217" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L217" s="5" t="n">
@@ -20183,7 +20183,7 @@
       </c>
       <c r="K218" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L218" s="5" t="n">
@@ -20255,7 +20255,7 @@
       </c>
       <c r="K219" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L219" s="5" t="n">
@@ -20327,7 +20327,7 @@
       </c>
       <c r="K220" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L220" s="5" t="n">
@@ -20399,7 +20399,7 @@
       </c>
       <c r="K221" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L221" s="5" t="n">
@@ -20471,7 +20471,7 @@
       </c>
       <c r="K222" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L222" s="5" t="n">
@@ -20543,7 +20543,7 @@
       </c>
       <c r="K223" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L223" s="5" t="n">
@@ -20615,7 +20615,7 @@
       </c>
       <c r="K224" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L224" s="5" t="n">
@@ -20687,7 +20687,7 @@
       </c>
       <c r="K225" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L225" s="5" t="n">
@@ -20759,7 +20759,7 @@
       </c>
       <c r="K226" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L226" s="5" t="n">
@@ -20831,7 +20831,7 @@
       </c>
       <c r="K227" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L227" s="5" t="n">
@@ -20903,7 +20903,7 @@
       </c>
       <c r="K228" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L228" s="5" t="n">
@@ -20975,7 +20975,7 @@
       </c>
       <c r="K229" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L229" s="5" t="n">
@@ -21047,7 +21047,7 @@
       </c>
       <c r="K230" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L230" s="5" t="n">
@@ -21119,7 +21119,7 @@
       </c>
       <c r="K231" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L231" s="5" t="n">
@@ -21191,7 +21191,7 @@
       </c>
       <c r="K232" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L232" s="5" t="n">
@@ -21263,7 +21263,7 @@
       </c>
       <c r="K233" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L233" s="5" t="n">
@@ -21335,7 +21335,7 @@
       </c>
       <c r="K234" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L234" s="5" t="n">
@@ -21407,7 +21407,7 @@
       </c>
       <c r="K235" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L235" s="5" t="n">
@@ -21479,7 +21479,7 @@
       </c>
       <c r="K236" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L236" s="5" t="n">
@@ -21551,7 +21551,7 @@
       </c>
       <c r="K237" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L237" s="5" t="n">
@@ -21623,7 +21623,7 @@
       </c>
       <c r="K238" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L238" s="5" t="n">
@@ -21695,7 +21695,7 @@
       </c>
       <c r="K239" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L239" s="5" t="n">
@@ -21767,7 +21767,7 @@
       </c>
       <c r="K240" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L240" s="5" t="n">
@@ -21839,7 +21839,7 @@
       </c>
       <c r="K241" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L241" s="5" t="n">
@@ -21911,7 +21911,7 @@
       </c>
       <c r="K242" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L242" s="5" t="n">
@@ -21983,7 +21983,7 @@
       </c>
       <c r="K243" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L243" s="5" t="n">
@@ -22055,7 +22055,7 @@
       </c>
       <c r="K244" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L244" s="5" t="n">
@@ -22127,7 +22127,7 @@
       </c>
       <c r="K245" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L245" s="5" t="n">
@@ -22199,7 +22199,7 @@
       </c>
       <c r="K246" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L246" s="5" t="n">
@@ -22271,7 +22271,7 @@
       </c>
       <c r="K247" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L247" s="5" t="n">
@@ -22343,7 +22343,7 @@
       </c>
       <c r="K248" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L248" s="5" t="n">
@@ -22415,7 +22415,7 @@
       </c>
       <c r="K249" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L249" s="5" t="n">
@@ -22487,7 +22487,7 @@
       </c>
       <c r="K250" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L250" s="5" t="n">
@@ -22559,7 +22559,7 @@
       </c>
       <c r="K251" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L251" s="5" t="n">
@@ -22631,7 +22631,7 @@
       </c>
       <c r="K252" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L252" s="5" t="n">
@@ -22703,7 +22703,7 @@
       </c>
       <c r="K253" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L253" s="5" t="n">
@@ -22775,7 +22775,7 @@
       </c>
       <c r="K254" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L254" s="5" t="n">
@@ -22847,7 +22847,7 @@
       </c>
       <c r="K255" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L255" s="5" t="n">
@@ -22919,7 +22919,7 @@
       </c>
       <c r="K256" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L256" s="5" t="n">
@@ -22991,7 +22991,7 @@
       </c>
       <c r="K257" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L257" s="5" t="n">
@@ -23063,7 +23063,7 @@
       </c>
       <c r="K258" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L258" s="5" t="n">
@@ -23135,7 +23135,7 @@
       </c>
       <c r="K259" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L259" s="5" t="n">
@@ -23207,7 +23207,7 @@
       </c>
       <c r="K260" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L260" s="5" t="n">
@@ -23279,7 +23279,7 @@
       </c>
       <c r="K261" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L261" s="5" t="n">
@@ -23351,7 +23351,7 @@
       </c>
       <c r="K262" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L262" s="5" t="n">
@@ -23423,7 +23423,7 @@
       </c>
       <c r="K263" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L263" s="5" t="n">
@@ -23495,7 +23495,7 @@
       </c>
       <c r="K264" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L264" s="5" t="n">
@@ -23567,7 +23567,7 @@
       </c>
       <c r="K265" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L265" s="5" t="n">
@@ -23639,7 +23639,7 @@
       </c>
       <c r="K266" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L266" s="5" t="n">
@@ -23711,7 +23711,7 @@
       </c>
       <c r="K267" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L267" s="5" t="n">
@@ -23783,7 +23783,7 @@
       </c>
       <c r="K268" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L268" s="5" t="n">
@@ -23855,7 +23855,7 @@
       </c>
       <c r="K269" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L269" s="5" t="n">
@@ -23927,7 +23927,7 @@
       </c>
       <c r="K270" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L270" s="5" t="n">
@@ -23999,7 +23999,7 @@
       </c>
       <c r="K271" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L271" s="5" t="n">
@@ -24071,7 +24071,7 @@
       </c>
       <c r="K272" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L272" s="5" t="n">
@@ -24143,7 +24143,7 @@
       </c>
       <c r="K273" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L273" s="5" t="n">
@@ -24215,7 +24215,7 @@
       </c>
       <c r="K274" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L274" s="5" t="n">
@@ -24287,7 +24287,7 @@
       </c>
       <c r="K275" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L275" s="5" t="n">
@@ -24359,7 +24359,7 @@
       </c>
       <c r="K276" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L276" s="5" t="n">
@@ -24431,7 +24431,7 @@
       </c>
       <c r="K277" s="2" t="inlineStr">
         <is>
-          <t>Repo (di vay)</t>
+          <t>Cho vay bond</t>
         </is>
       </c>
       <c r="L277" s="5" t="n">

</xml_diff>